<commit_message>
add studies of Chinese ancient civilization
</commit_message>
<xml_diff>
--- a/bill/living_payment.xlsx
+++ b/bill/living_payment.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="23127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="23231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\alantop_dir\alantop_data\alantop_git\github\bill\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AD0D777-FB25-42F2-868F-2821FF23DD09}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF7A73B6-D938-4FF9-925D-C0E12E316433}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="浦东" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="76">
   <si>
     <t>金额</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -291,6 +291,46 @@
   </si>
   <si>
     <t>使用规则</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>天燃气</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>最后付费</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>备注</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>居雯静支付</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>电费</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>和瑞雅苑天燃气</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>客户编号：50899535</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>张支付宝支付 支付日期2020.10.11，支付宝优惠0.5</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>支付日期10.11 张掌上生活 优惠1元</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>支付</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -426,7 +466,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -492,6 +532,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -773,25 +814,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G22"/>
-  <sheetFormatPr defaultRowHeight="17.399999999999999" customHeight="1" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:G23"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="17.45" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.44140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="32.88671875" style="7" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.44140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.88671875" style="7" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.21875" style="14" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="25.5546875" style="7" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="25.5546875" style="7" customWidth="1"/>
-    <col min="8" max="8" width="8.109375" style="7" customWidth="1"/>
-    <col min="9" max="9" width="8.88671875" style="7"/>
+    <col min="1" max="1" width="11.5" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.875" style="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.5" style="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.875" style="7" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.25" style="14" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="50.25" style="7" customWidth="1"/>
+    <col min="7" max="7" width="25.5" style="7" customWidth="1"/>
+    <col min="8" max="8" width="8.125" style="7" customWidth="1"/>
+    <col min="9" max="9" width="8.875" style="7"/>
     <col min="10" max="10" width="13" style="7" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.88671875" style="7"/>
-    <col min="12" max="12" width="12.77734375" style="7" bestFit="1" customWidth="1"/>
-    <col min="13" max="16384" width="8.88671875" style="7"/>
+    <col min="11" max="11" width="8.875" style="7"/>
+    <col min="12" max="12" width="12.75" style="7" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="8.875" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="5" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" s="5" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
         <v>13</v>
       </c>
@@ -814,7 +855,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="6">
         <v>44026</v>
       </c>
@@ -834,7 +875,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="6">
         <v>44043</v>
       </c>
@@ -854,7 +895,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="6">
         <v>44043</v>
       </c>
@@ -874,7 +915,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="6">
         <v>44043</v>
       </c>
@@ -891,7 +932,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="6">
         <v>44043</v>
       </c>
@@ -911,7 +952,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="6">
         <v>44043</v>
       </c>
@@ -931,7 +972,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="6">
         <v>44057</v>
       </c>
@@ -948,7 +989,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="6">
         <v>44074</v>
       </c>
@@ -962,7 +1003,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="6">
         <v>44074</v>
       </c>
@@ -982,7 +1023,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="6">
         <v>44054</v>
       </c>
@@ -1002,7 +1043,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="6">
         <v>44053</v>
       </c>
@@ -1019,7 +1060,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="6">
         <v>44074</v>
       </c>
@@ -1039,7 +1080,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="6">
         <v>44074</v>
       </c>
@@ -1059,7 +1100,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="6">
         <v>44087</v>
       </c>
@@ -1076,7 +1117,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:7" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B17" s="7" t="s">
         <v>45</v>
       </c>
@@ -1084,7 +1125,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="7" t="s">
         <v>46</v>
       </c>
@@ -1092,7 +1133,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:7" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="6">
         <v>44104</v>
       </c>
@@ -1112,7 +1153,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:7" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="6">
         <v>44104</v>
       </c>
@@ -1123,7 +1164,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:7" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="6">
         <v>44104</v>
       </c>
@@ -1143,7 +1184,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:7" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="6">
         <v>44104</v>
       </c>
@@ -1158,6 +1199,23 @@
       </c>
       <c r="F22" s="7" t="s">
         <v>55</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="6">
+        <v>44116</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="C23" s="8">
+        <v>99</v>
+      </c>
+      <c r="E23" s="14">
+        <v>1</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -1169,9 +1227,73 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7CB4EC01-2964-4381-B658-6411095BFCC5}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="11.125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.25" customWidth="1"/>
+    <col min="7" max="7" width="32.625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>67</v>
+      </c>
+      <c r="D1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1" t="s">
+        <v>57</v>
+      </c>
+      <c r="H1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2" s="29">
+        <v>44144</v>
+      </c>
+      <c r="B2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C2">
+        <v>39</v>
+      </c>
+      <c r="D2" s="29">
+        <v>44114</v>
+      </c>
+      <c r="E2" t="s">
+        <v>69</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" s="29">
+        <v>44135</v>
+      </c>
+      <c r="B3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C3">
+        <v>63.8</v>
+      </c>
+      <c r="F3" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="G3" t="s">
+        <v>74</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -1181,14 +1303,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{816541AC-AEEC-440E-9B2B-A42B017C90F5}">
   <dimension ref="A1:E14"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="11.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.77734375" style="23" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.75" style="23" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="17.399999999999999" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="18" x14ac:dyDescent="0.2">
       <c r="A1" s="24" t="s">
         <v>60</v>
       </c>
@@ -1203,7 +1325,7 @@
       </c>
       <c r="E1" s="24"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="26">
         <v>1</v>
       </c>
@@ -1218,7 +1340,7 @@
       </c>
       <c r="E2" s="10"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="26">
         <v>2</v>
       </c>
@@ -1231,7 +1353,7 @@
       </c>
       <c r="E3" s="12"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="26">
         <v>3</v>
       </c>
@@ -1244,7 +1366,7 @@
       </c>
       <c r="E4" s="10"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="26">
         <v>4</v>
       </c>
@@ -1257,7 +1379,7 @@
       </c>
       <c r="E5" s="10"/>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="26">
         <v>5</v>
       </c>
@@ -1270,14 +1392,14 @@
       </c>
       <c r="E6" s="10"/>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="27"/>
       <c r="B7" s="15"/>
       <c r="C7" s="15"/>
       <c r="D7" s="19"/>
       <c r="E7" s="15"/>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="26">
         <v>1</v>
       </c>
@@ -1292,7 +1414,7 @@
       </c>
       <c r="E8" s="10"/>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="26">
         <v>2</v>
       </c>
@@ -1305,7 +1427,7 @@
       </c>
       <c r="E9" s="10"/>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="26">
         <v>3</v>
       </c>
@@ -1320,45 +1442,51 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="26">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" s="27"/>
+      <c r="B11" s="7"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="21"/>
+      <c r="E11" s="7"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" s="26">
+        <v>1</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" s="10"/>
+      <c r="D12" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="E12" s="10"/>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" s="26">
+        <v>2</v>
+      </c>
+      <c r="B13" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="C13" s="16"/>
+      <c r="D13" s="22" t="s">
+        <v>72</v>
+      </c>
+      <c r="E13" s="16"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" s="26">
         <v>4</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B14" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="C11" s="10"/>
-      <c r="D11" s="17" t="s">
+      <c r="C14" s="10"/>
+      <c r="D14" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="E11" s="10"/>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="27"/>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="21"/>
-      <c r="E12" s="7"/>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="26">
-        <v>1</v>
-      </c>
-      <c r="B13" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="C13" s="10"/>
-      <c r="D13" s="17" t="s">
-        <v>34</v>
-      </c>
-      <c r="E13" s="10"/>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="26"/>
-      <c r="B14" s="16"/>
-      <c r="C14" s="16"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="16"/>
+      <c r="E14" s="10"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -1370,14 +1498,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDE900A6-FCDE-4A42-A762-67519E3C38A8}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="26" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="28" t="s">
         <v>62</v>
       </c>
@@ -1391,7 +1519,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>63</v>
       </c>

</xml_diff>